<commit_message>
Update 703634 - MSCI Switzerland 20_35 Index .xlsx
</commit_message>
<xml_diff>
--- a/data/703634 - MSCI Switzerland 20_35 Index .xlsx
+++ b/data/703634 - MSCI Switzerland 20_35 Index .xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4673" uniqueCount="4672">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4697" uniqueCount="4696">
   <si>
     <t>Index Level:</t>
   </si>
@@ -14027,6 +14027,78 @@
   </si>
   <si>
     <t>2026-03-27</t>
+  </si>
+  <si>
+    <t>2026-03-30</t>
+  </si>
+  <si>
+    <t>2026-03-31</t>
+  </si>
+  <si>
+    <t>2026-04-01</t>
+  </si>
+  <si>
+    <t>2026-04-02</t>
+  </si>
+  <si>
+    <t>2026-04-03</t>
+  </si>
+  <si>
+    <t>2026-04-06</t>
+  </si>
+  <si>
+    <t>2026-04-07</t>
+  </si>
+  <si>
+    <t>2026-04-08</t>
+  </si>
+  <si>
+    <t>2026-04-09</t>
+  </si>
+  <si>
+    <t>2026-04-10</t>
+  </si>
+  <si>
+    <t>2026-04-13</t>
+  </si>
+  <si>
+    <t>2026-04-14</t>
+  </si>
+  <si>
+    <t>2026-04-15</t>
+  </si>
+  <si>
+    <t>2026-04-16</t>
+  </si>
+  <si>
+    <t>2026-04-17</t>
+  </si>
+  <si>
+    <t>2026-04-20</t>
+  </si>
+  <si>
+    <t>2026-04-21</t>
+  </si>
+  <si>
+    <t>2026-04-22</t>
+  </si>
+  <si>
+    <t>2026-04-23</t>
+  </si>
+  <si>
+    <t>2026-04-24</t>
+  </si>
+  <si>
+    <t>2026-04-27</t>
+  </si>
+  <si>
+    <t>2026-04-28</t>
+  </si>
+  <si>
+    <t>2026-04-29</t>
+  </si>
+  <si>
+    <t>2026-04-30</t>
   </si>
 </sst>
 </file>
@@ -14412,7 +14484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:E4657"/>
+  <dimension ref="A3:E4681"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -51705,6 +51777,198 @@
         <v>3137.6098</v>
       </c>
     </row>
+    <row r="4658" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4658" t="s">
+        <v>4672</v>
+      </c>
+      <c r="B4658">
+        <v>3149.161191</v>
+      </c>
+    </row>
+    <row r="4659" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4659" t="s">
+        <v>4673</v>
+      </c>
+      <c r="B4659">
+        <v>3163.758015</v>
+      </c>
+    </row>
+    <row r="4660" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4660" t="s">
+        <v>4674</v>
+      </c>
+      <c r="B4660">
+        <v>3259.918571</v>
+      </c>
+    </row>
+    <row r="4661" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4661" t="s">
+        <v>4675</v>
+      </c>
+      <c r="B4661">
+        <v>3233.731824</v>
+      </c>
+    </row>
+    <row r="4662" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4662" t="s">
+        <v>4676</v>
+      </c>
+      <c r="B4662">
+        <v>3233.731824</v>
+      </c>
+    </row>
+    <row r="4663" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4663" t="s">
+        <v>4677</v>
+      </c>
+      <c r="B4663">
+        <v>3237.784373</v>
+      </c>
+    </row>
+    <row r="4664" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4664" t="s">
+        <v>4678</v>
+      </c>
+      <c r="B4664">
+        <v>3180.836972</v>
+      </c>
+    </row>
+    <row r="4665" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4665" t="s">
+        <v>4679</v>
+      </c>
+      <c r="B4665">
+        <v>3310.083523</v>
+      </c>
+    </row>
+    <row r="4666" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4666" t="s">
+        <v>4680</v>
+      </c>
+      <c r="B4666">
+        <v>3313.477489</v>
+      </c>
+    </row>
+    <row r="4667" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4667" t="s">
+        <v>4681</v>
+      </c>
+      <c r="B4667">
+        <v>3334.626311</v>
+      </c>
+    </row>
+    <row r="4668" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4668" t="s">
+        <v>4682</v>
+      </c>
+      <c r="B4668">
+        <v>3332.261614</v>
+      </c>
+    </row>
+    <row r="4669" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4669" t="s">
+        <v>4683</v>
+      </c>
+      <c r="B4669">
+        <v>3397.647126</v>
+      </c>
+    </row>
+    <row r="4670" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4670" t="s">
+        <v>4684</v>
+      </c>
+      <c r="B4670">
+        <v>3379.820984</v>
+      </c>
+    </row>
+    <row r="4671" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4671" t="s">
+        <v>4685</v>
+      </c>
+      <c r="B4671">
+        <v>3354.913363</v>
+      </c>
+    </row>
+    <row r="4672" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4672" t="s">
+        <v>4686</v>
+      </c>
+      <c r="B4672">
+        <v>3444.608845</v>
+      </c>
+    </row>
+    <row r="4673" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4673" t="s">
+        <v>4687</v>
+      </c>
+      <c r="B4673">
+        <v>3421.187668</v>
+      </c>
+    </row>
+    <row r="4674" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4674" t="s">
+        <v>4688</v>
+      </c>
+      <c r="B4674">
+        <v>3382.204908</v>
+      </c>
+    </row>
+    <row r="4675" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4675" t="s">
+        <v>4689</v>
+      </c>
+      <c r="B4675">
+        <v>3347.54564</v>
+      </c>
+    </row>
+    <row r="4676" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4676" t="s">
+        <v>4690</v>
+      </c>
+      <c r="B4676">
+        <v>3391.450663</v>
+      </c>
+    </row>
+    <row r="4677" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4677" t="s">
+        <v>4691</v>
+      </c>
+      <c r="B4677">
+        <v>3360.723365</v>
+      </c>
+    </row>
+    <row r="4678" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4678" t="s">
+        <v>4692</v>
+      </c>
+      <c r="B4678">
+        <v>3364.171043</v>
+      </c>
+    </row>
+    <row r="4679" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4679" t="s">
+        <v>4693</v>
+      </c>
+      <c r="B4679">
+        <v>3332.22523</v>
+      </c>
+    </row>
+    <row r="4680" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4680" t="s">
+        <v>4694</v>
+      </c>
+      <c r="B4680">
+        <v>3307.086604</v>
+      </c>
+    </row>
+    <row r="4681" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4681" t="s">
+        <v>4695</v>
+      </c>
+      <c r="B4681">
+        <v>3371.191496</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>